<commit_message>
adds diagnostics and revised scaa rtmb model
</commit_message>
<xml_diff>
--- a/materials/2025-11-04/data/floundah_agecomps.xlsx
+++ b/materials/2025-11-04/data/floundah_agecomps.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gfay/courses/mar580-advpopmod-f25/materials/2025-10-14/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gfay/courses/mar580-advpopmod-f25/materials/2025-11-04/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{766A8E8B-5710-B245-97DD-79761F22D0AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A936E105-BF79-7E44-AFDB-7DC58C94B1BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13080" yWindow="500" windowWidth="27240" windowHeight="17180" activeTab="1" xr2:uid="{9AB6F010-7017-6646-8DC6-C46A0D642F05}"/>
+    <workbookView xWindow="2160" yWindow="740" windowWidth="27240" windowHeight="17180" xr2:uid="{9AB6F010-7017-6646-8DC6-C46A0D642F05}"/>
   </bookViews>
   <sheets>
     <sheet name="fishery" sheetId="1" r:id="rId1"/>
@@ -440,16 +440,16 @@
         <v>1963</v>
       </c>
       <c r="B2" s="1">
-        <v>0.33985082167401198</v>
+        <v>0.35</v>
       </c>
       <c r="C2" s="1">
-        <v>0.42676093010081123</v>
+        <v>0.45</v>
       </c>
       <c r="D2" s="1">
-        <v>0.13494483417677502</v>
+        <v>0.08</v>
       </c>
       <c r="E2" s="1">
-        <v>9.8443414048401637E-2</v>
+        <v>0.12</v>
       </c>
       <c r="F2" s="1">
         <v>0</v>
@@ -460,19 +460,19 @@
         <v>1964</v>
       </c>
       <c r="B3" s="1">
-        <v>0.2699391320188686</v>
+        <v>0.2</v>
       </c>
       <c r="C3" s="1">
-        <v>0.42305070749053353</v>
+        <v>0.43</v>
       </c>
       <c r="D3" s="1">
-        <v>0.21730402680544314</v>
+        <v>0.24</v>
       </c>
       <c r="E3" s="1">
-        <v>5.7113172261650635E-2</v>
+        <v>0.09</v>
       </c>
       <c r="F3" s="1">
-        <v>3.2592961423504097E-2</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -480,19 +480,19 @@
         <v>1965</v>
       </c>
       <c r="B4" s="1">
-        <v>0.15905805398302045</v>
+        <v>0.2</v>
       </c>
       <c r="C4" s="1">
-        <v>0.43068001768018022</v>
+        <v>0.42</v>
       </c>
       <c r="D4" s="1">
-        <v>0.22224503297769424</v>
+        <v>0.22</v>
       </c>
       <c r="E4" s="1">
-        <v>8.7643574045034214E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F4" s="1">
-        <v>0.10037332131407084</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -500,19 +500,19 @@
         <v>1966</v>
       </c>
       <c r="B5" s="1">
-        <v>0.1107320923548073</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="C5" s="1">
-        <v>0.38702559947010667</v>
+        <v>0.39</v>
       </c>
       <c r="D5" s="1">
-        <v>0.34687275232414383</v>
+        <v>0.33</v>
       </c>
       <c r="E5" s="1">
-        <v>0.12033874368631112</v>
+        <v>0.12</v>
       </c>
       <c r="F5" s="1">
-        <v>3.5030812164631109E-2</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -520,19 +520,19 @@
         <v>1967</v>
       </c>
       <c r="B6" s="1">
-        <v>0.35510015506049608</v>
+        <v>0.4</v>
       </c>
       <c r="C6" s="1">
-        <v>0.21578166501855786</v>
+        <v>0.25</v>
       </c>
       <c r="D6" s="1">
-        <v>0.21664280104152125</v>
+        <v>0.24</v>
       </c>
       <c r="E6" s="1">
-        <v>0.12266181302644243</v>
+        <v>0.09</v>
       </c>
       <c r="F6" s="1">
-        <v>8.9813565852982391E-2</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -540,19 +540,19 @@
         <v>1968</v>
       </c>
       <c r="B7" s="1">
-        <v>0.38157600255169127</v>
+        <v>0.37</v>
       </c>
       <c r="C7" s="1">
-        <v>0.4602949364842433</v>
+        <v>0.46</v>
       </c>
       <c r="D7" s="1">
-        <v>9.4096920329966693E-2</v>
+        <v>0.08</v>
       </c>
       <c r="E7" s="1">
-        <v>6.0234730680804503E-2</v>
+        <v>0.09</v>
       </c>
       <c r="F7" s="1">
-        <v>3.7974099532941397E-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -560,19 +560,19 @@
         <v>1969</v>
       </c>
       <c r="B8" s="1">
-        <v>0.14273608056867634</v>
+        <v>0.13</v>
       </c>
       <c r="C8" s="1">
-        <v>0.51150297660976607</v>
+        <v>0.45</v>
       </c>
       <c r="D8" s="1">
-        <v>0.23458566775579201</v>
+        <v>0.26</v>
       </c>
       <c r="E8" s="1">
-        <v>3.1730897104148649E-2</v>
+        <v>0.06</v>
       </c>
       <c r="F8" s="1">
-        <v>7.9444377961616852E-2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -580,19 +580,19 @@
         <v>1970</v>
       </c>
       <c r="B9" s="1">
-        <v>0.3279946809165763</v>
+        <v>0.39</v>
       </c>
       <c r="C9" s="1">
-        <v>0.25415068517836903</v>
+        <v>0.22</v>
       </c>
       <c r="D9" s="1">
-        <v>0.25467078805870419</v>
+        <v>0.27</v>
       </c>
       <c r="E9" s="1">
-        <v>6.5951840511741397E-2</v>
+        <v>0.01</v>
       </c>
       <c r="F9" s="1">
-        <v>9.7232005334608962E-2</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -600,16 +600,16 @@
         <v>1971</v>
       </c>
       <c r="B10" s="1">
-        <v>0.41844925859611964</v>
+        <v>0.49</v>
       </c>
       <c r="C10" s="1">
-        <v>0.4421840772755728</v>
+        <v>0.33</v>
       </c>
       <c r="D10" s="1">
-        <v>7.278313570325308E-2</v>
+        <v>0.12</v>
       </c>
       <c r="E10" s="1">
-        <v>6.658352842505455E-2</v>
+        <v>0.06</v>
       </c>
       <c r="F10" s="1">
         <v>0</v>
@@ -620,16 +620,16 @@
         <v>1972</v>
       </c>
       <c r="B11" s="1">
-        <v>0.13908104121138443</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="C11" s="1">
-        <v>0.68788208530906481</v>
+        <v>0.67</v>
       </c>
       <c r="D11" s="1">
-        <v>0.15376623010526555</v>
+        <v>0.18</v>
       </c>
       <c r="E11" s="1">
-        <v>1.9270643374285107E-2</v>
+        <v>0.01</v>
       </c>
       <c r="F11" s="1">
         <v>0</v>
@@ -640,19 +640,19 @@
         <v>1973</v>
       </c>
       <c r="B12" s="1">
-        <v>0.37741597860028769</v>
+        <v>0.34</v>
       </c>
       <c r="C12" s="1">
-        <v>0.2661404833845214</v>
+        <v>0.32</v>
       </c>
       <c r="D12" s="1">
-        <v>0.27200576658867437</v>
+        <v>0.24</v>
       </c>
       <c r="E12" s="1">
-        <v>6.5477792113918604E-2</v>
+        <v>0.1</v>
       </c>
       <c r="F12" s="1">
-        <v>1.8959979312597963E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -660,16 +660,16 @@
         <v>1974</v>
       </c>
       <c r="B13" s="1">
-        <v>0.34677660239337177</v>
+        <v>0.36</v>
       </c>
       <c r="C13" s="1">
-        <v>0.49249396189207029</v>
+        <v>0.5</v>
       </c>
       <c r="D13" s="1">
-        <v>8.4527633072781369E-2</v>
+        <v>0.06</v>
       </c>
       <c r="E13" s="1">
-        <v>7.6201802641776534E-2</v>
+        <v>0.08</v>
       </c>
       <c r="F13" s="1">
         <v>0</v>
@@ -680,16 +680,16 @@
         <v>1975</v>
       </c>
       <c r="B14" s="1">
-        <v>0.14731874313609464</v>
+        <v>0.25</v>
       </c>
       <c r="C14" s="1">
-        <v>0.5768744189385967</v>
+        <v>0.5</v>
       </c>
       <c r="D14" s="1">
-        <v>0.24492572261172105</v>
+        <v>0.21</v>
       </c>
       <c r="E14" s="1">
-        <v>3.0881115313587601E-2</v>
+        <v>0.04</v>
       </c>
       <c r="F14" s="1">
         <v>0</v>
@@ -700,19 +700,19 @@
         <v>1976</v>
       </c>
       <c r="B15" s="1">
-        <v>0.49941815556334163</v>
+        <v>0.48</v>
       </c>
       <c r="C15" s="1">
-        <v>0.17837557233933923</v>
+        <v>0.16</v>
       </c>
       <c r="D15" s="1">
-        <v>0.18522216964419272</v>
+        <v>0.22</v>
       </c>
       <c r="E15" s="1">
-        <v>6.1024575407333755E-2</v>
+        <v>0.06</v>
       </c>
       <c r="F15" s="1">
-        <v>7.5959527045792674E-2</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -720,19 +720,19 @@
         <v>1977</v>
       </c>
       <c r="B16" s="1">
-        <v>0.34710740875664681</v>
+        <v>0.35</v>
       </c>
       <c r="C16" s="1">
-        <v>0.48128801834852653</v>
+        <v>0.52</v>
       </c>
       <c r="D16" s="1">
-        <v>5.9826300267630021E-2</v>
+        <v>0.03</v>
       </c>
       <c r="E16" s="1">
-        <v>4.2317499131286358E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F16" s="1">
-        <v>6.9460773495910288E-2</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -740,19 +740,19 @@
         <v>1978</v>
       </c>
       <c r="B17" s="1">
-        <v>0.29950338698554829</v>
+        <v>0.26</v>
       </c>
       <c r="C17" s="1">
-        <v>0.44034250825926036</v>
+        <v>0.4</v>
       </c>
       <c r="D17" s="1">
-        <v>0.22099151253074961</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="E17" s="1">
-        <v>1.8042736531451446E-2</v>
+        <v>0.03</v>
       </c>
       <c r="F17" s="1">
-        <v>2.1119855692990352E-2</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -760,19 +760,19 @@
         <v>1979</v>
       </c>
       <c r="B18" s="1">
-        <v>0.44558911145197339</v>
+        <v>0.4</v>
       </c>
       <c r="C18" s="1">
-        <v>0.32192613306222034</v>
+        <v>0.32</v>
       </c>
       <c r="D18" s="1">
-        <v>0.17859968101973503</v>
+        <v>0.26</v>
       </c>
       <c r="E18" s="1">
-        <v>4.4234787601053947E-2</v>
+        <v>0.02</v>
       </c>
       <c r="F18" s="1">
-        <v>9.6502868650173435E-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -780,19 +780,19 @@
         <v>1980</v>
       </c>
       <c r="B19" s="1">
-        <v>0.28985267634268252</v>
+        <v>0.25</v>
       </c>
       <c r="C19" s="1">
-        <v>0.50288387490572117</v>
+        <v>0.54</v>
       </c>
       <c r="D19" s="1">
-        <v>0.1137797303158177</v>
+        <v>0.16</v>
       </c>
       <c r="E19" s="1">
-        <v>3.0522006423903243E-2</v>
+        <v>0</v>
       </c>
       <c r="F19" s="1">
-        <v>6.2961712011875393E-2</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -800,16 +800,16 @@
         <v>1981</v>
       </c>
       <c r="B20" s="1">
-        <v>0.2357686086702678</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="C20" s="1">
-        <v>0.46650834070534697</v>
+        <v>0.43</v>
       </c>
       <c r="D20" s="1">
-        <v>0.26037364772731331</v>
+        <v>0.25</v>
       </c>
       <c r="E20" s="1">
-        <v>3.7349402897072038E-2</v>
+        <v>0.04</v>
       </c>
       <c r="F20" s="1">
         <v>0</v>
@@ -820,16 +820,16 @@
         <v>1982</v>
       </c>
       <c r="B21" s="1">
-        <v>0.67096204391924719</v>
+        <v>0.62</v>
       </c>
       <c r="C21" s="1">
-        <v>0.17436635366273451</v>
+        <v>0.19</v>
       </c>
       <c r="D21" s="1">
-        <v>0.11551986814010547</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="E21" s="1">
-        <v>3.9151734277912652E-2</v>
+        <v>0.05</v>
       </c>
       <c r="F21" s="1">
         <v>0</v>
@@ -840,16 +840,16 @@
         <v>1983</v>
       </c>
       <c r="B22" s="1">
-        <v>0.15137341845796518</v>
+        <v>0.17</v>
       </c>
       <c r="C22" s="1">
-        <v>0.76154688949270888</v>
+        <v>0.77</v>
       </c>
       <c r="D22" s="1">
-        <v>6.5503655050652754E-2</v>
+        <v>0.04</v>
       </c>
       <c r="E22" s="1">
-        <v>2.157603699867313E-2</v>
+        <v>0.02</v>
       </c>
       <c r="F22" s="1">
         <v>0</v>
@@ -860,19 +860,19 @@
         <v>1984</v>
       </c>
       <c r="B23" s="1">
-        <v>0.22740054002877269</v>
+        <v>0.27</v>
       </c>
       <c r="C23" s="1">
-        <v>0.27073483621357641</v>
+        <v>0.22</v>
       </c>
       <c r="D23" s="1">
-        <v>0.44425319065232272</v>
+        <v>0.43</v>
       </c>
       <c r="E23" s="1">
-        <v>2.3461842285536702E-2</v>
+        <v>0.03</v>
       </c>
       <c r="F23" s="1">
-        <v>3.4149590819791409E-2</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
@@ -880,16 +880,16 @@
         <v>1985</v>
       </c>
       <c r="B24" s="1">
-        <v>0.49091647460314297</v>
+        <v>0.52</v>
       </c>
       <c r="C24" s="1">
-        <v>0.27718163078410663</v>
+        <v>0.21</v>
       </c>
       <c r="D24" s="1">
-        <v>0.12674315159695362</v>
+        <v>0.15</v>
       </c>
       <c r="E24" s="1">
-        <v>0.10515874301579681</v>
+        <v>0.12</v>
       </c>
       <c r="F24" s="1">
         <v>0</v>
@@ -900,19 +900,19 @@
         <v>1986</v>
       </c>
       <c r="B25" s="1">
-        <v>0.36335054887623303</v>
+        <v>0.33</v>
       </c>
       <c r="C25" s="1">
-        <v>0.43364912723578136</v>
+        <v>0.5</v>
       </c>
       <c r="D25" s="1">
-        <v>9.1874265888739079E-2</v>
+        <v>0.11</v>
       </c>
       <c r="E25" s="1">
-        <v>3.010407774445099E-2</v>
+        <v>0.01</v>
       </c>
       <c r="F25" s="1">
-        <v>8.1021980254795567E-2</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
@@ -920,19 +920,19 @@
         <v>1987</v>
       </c>
       <c r="B26" s="1">
-        <v>0.26571102012073056</v>
+        <v>0.26</v>
       </c>
       <c r="C26" s="1">
-        <v>0.43980972879857927</v>
+        <v>0.41</v>
       </c>
       <c r="D26" s="1">
-        <v>0.21091272154718527</v>
+        <v>0.21</v>
       </c>
       <c r="E26" s="1">
-        <v>2.8935648930086301E-2</v>
+        <v>0.03</v>
       </c>
       <c r="F26" s="1">
-        <v>5.4630880603418586E-2</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
@@ -940,19 +940,19 @@
         <v>1988</v>
       </c>
       <c r="B27" s="1">
-        <v>0.48027552828830355</v>
+        <v>0.5</v>
       </c>
       <c r="C27" s="1">
-        <v>0.29197457925867909</v>
+        <v>0.3</v>
       </c>
       <c r="D27" s="1">
-        <v>0.14326848195303429</v>
+        <v>0.12</v>
       </c>
       <c r="E27" s="1">
-        <v>4.2885887733787043E-2</v>
+        <v>0.04</v>
       </c>
       <c r="F27" s="1">
-        <v>4.1595522766195936E-2</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
@@ -960,19 +960,19 @@
         <v>1989</v>
       </c>
       <c r="B28" s="1">
-        <v>0.25988574276164755</v>
+        <v>0.3</v>
       </c>
       <c r="C28" s="1">
-        <v>0.54638680157759734</v>
+        <v>0.48</v>
       </c>
       <c r="D28" s="1">
-        <v>0.10768826602756877</v>
+        <v>0.09</v>
       </c>
       <c r="E28" s="1">
-        <v>3.7182153656092502E-2</v>
+        <v>0.03</v>
       </c>
       <c r="F28" s="1">
-        <v>4.8857035977093899E-2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
@@ -980,16 +980,16 @@
         <v>1990</v>
       </c>
       <c r="B29" s="1">
-        <v>0.34853804765072299</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="C29" s="1">
-        <v>0.37241713864064746</v>
+        <v>0.44</v>
       </c>
       <c r="D29" s="1">
-        <v>0.25361486930761751</v>
+        <v>0.24</v>
       </c>
       <c r="E29" s="1">
-        <v>2.5429944401011938E-2</v>
+        <v>0.04</v>
       </c>
       <c r="F29" s="1">
         <v>0</v>
@@ -1000,16 +1000,16 @@
         <v>1991</v>
       </c>
       <c r="B30" s="1">
-        <v>0.3884334708341739</v>
+        <v>0.38</v>
       </c>
       <c r="C30" s="1">
-        <v>0.4380613815539684</v>
+        <v>0.46</v>
       </c>
       <c r="D30" s="1">
-        <v>0.12391665834778737</v>
+        <v>0.11</v>
       </c>
       <c r="E30" s="1">
-        <v>4.9588489264070321E-2</v>
+        <v>0.05</v>
       </c>
       <c r="F30" s="1">
         <v>0</v>
@@ -1020,19 +1020,19 @@
         <v>1992</v>
       </c>
       <c r="B31" s="1">
-        <v>0.48067525191969557</v>
+        <v>0.51</v>
       </c>
       <c r="C31" s="1">
-        <v>0.30481672774857715</v>
+        <v>0.27</v>
       </c>
       <c r="D31" s="1">
-        <v>0.1388227182835855</v>
+        <v>0.13</v>
       </c>
       <c r="E31" s="1">
-        <v>1.9634500022693891E-2</v>
+        <v>0</v>
       </c>
       <c r="F31" s="1">
-        <v>5.6050802025447988E-2</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
@@ -1040,16 +1040,16 @@
         <v>1993</v>
       </c>
       <c r="B32" s="1">
-        <v>0.26057535533563897</v>
+        <v>0.23</v>
       </c>
       <c r="C32" s="1">
-        <v>0.59899574221974927</v>
+        <v>0.61</v>
       </c>
       <c r="D32" s="1">
-        <v>0.10879044129481516</v>
+        <v>0.12</v>
       </c>
       <c r="E32" s="1">
-        <v>3.1638461149796619E-2</v>
+        <v>0.04</v>
       </c>
       <c r="F32" s="1">
         <v>0</v>
@@ -1060,16 +1060,16 @@
         <v>1994</v>
       </c>
       <c r="B33" s="1">
-        <v>0.13863331320934458</v>
+        <v>0.09</v>
       </c>
       <c r="C33" s="1">
-        <v>0.43244164463030399</v>
+        <v>0.44</v>
       </c>
       <c r="D33" s="1">
-        <v>0.3877724000112629</v>
+        <v>0.42</v>
       </c>
       <c r="E33" s="1">
-        <v>4.1152642149088606E-2</v>
+        <v>0.05</v>
       </c>
       <c r="F33" s="1">
         <v>0</v>
@@ -1080,16 +1080,16 @@
         <v>1995</v>
       </c>
       <c r="B34" s="1">
-        <v>0.37918363895439655</v>
+        <v>0.36</v>
       </c>
       <c r="C34" s="1">
-        <v>0.22993058950206718</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="D34" s="1">
-        <v>0.24037922605713175</v>
+        <v>0.22</v>
       </c>
       <c r="E34" s="1">
-        <v>0.15050654548640463</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="F34" s="1">
         <v>0</v>
@@ -1100,19 +1100,19 @@
         <v>1996</v>
       </c>
       <c r="B35" s="1">
-        <v>0.17330885546366223</v>
+        <v>0.19</v>
       </c>
       <c r="C35" s="1">
-        <v>0.47688304430610839</v>
+        <v>0.54</v>
       </c>
       <c r="D35" s="1">
-        <v>0.12596279626289811</v>
+        <v>0.11</v>
       </c>
       <c r="E35" s="1">
-        <v>9.4056422168701317E-2</v>
+        <v>0.06</v>
       </c>
       <c r="F35" s="1">
-        <v>0.12978888179862991</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
@@ -1120,19 +1120,19 @@
         <v>1997</v>
       </c>
       <c r="B36" s="1">
-        <v>0.1320878634094303</v>
+        <v>0.17</v>
       </c>
       <c r="C36" s="1">
-        <v>0.28825769534164908</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="D36" s="1">
-        <v>0.38323020517147582</v>
+        <v>0.3</v>
       </c>
       <c r="E36" s="1">
-        <v>6.5570299642944391E-2</v>
+        <v>0.08</v>
       </c>
       <c r="F36" s="1">
-        <v>0.1308539364345005</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
@@ -1140,19 +1140,19 @@
         <v>1998</v>
       </c>
       <c r="B37" s="1">
-        <v>0.2257196933951649</v>
+        <v>0.2</v>
       </c>
       <c r="C37" s="1">
-        <v>0.23116235344918867</v>
+        <v>0.27</v>
       </c>
       <c r="D37" s="1">
-        <v>0.24259928287568111</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="E37" s="1">
-        <v>0.20197260639426654</v>
+        <v>0.15</v>
       </c>
       <c r="F37" s="1">
-        <v>9.8546063885698865E-2</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
@@ -1160,19 +1160,19 @@
         <v>1999</v>
       </c>
       <c r="B38" s="1">
-        <v>0.24321212139901072</v>
+        <v>0.2</v>
       </c>
       <c r="C38" s="1">
-        <v>0.37255128573293367</v>
+        <v>0.34</v>
       </c>
       <c r="D38" s="1">
-        <v>0.15278123991462916</v>
+        <v>0.17</v>
       </c>
       <c r="E38" s="1">
-        <v>0.1107194992364892</v>
+        <v>0.18</v>
       </c>
       <c r="F38" s="1">
-        <v>0.12073585371693729</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
@@ -1180,19 +1180,19 @@
         <v>2000</v>
       </c>
       <c r="B39" s="1">
-        <v>0.13879463464915021</v>
+        <v>0.12</v>
       </c>
       <c r="C39" s="1">
-        <v>0.41698530982716919</v>
+        <v>0.45</v>
       </c>
       <c r="D39" s="1">
-        <v>0.25348572806420688</v>
+        <v>0.24</v>
       </c>
       <c r="E39" s="1">
-        <v>6.8634189978571028E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F39" s="1">
-        <v>0.12210013748090265</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
@@ -1200,19 +1200,19 @@
         <v>2001</v>
       </c>
       <c r="B40" s="1">
-        <v>0.19171080461930334</v>
+        <v>0.15</v>
       </c>
       <c r="C40" s="1">
-        <v>0.26347285690261146</v>
+        <v>0.21</v>
       </c>
       <c r="D40" s="1">
-        <v>0.30822305639769326</v>
+        <v>0.31</v>
       </c>
       <c r="E40" s="1">
-        <v>0.13864269907605367</v>
+        <v>0.18</v>
       </c>
       <c r="F40" s="1">
-        <v>9.7950583004338343E-2</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
@@ -1220,19 +1220,19 @@
         <v>2002</v>
       </c>
       <c r="B41" s="1">
-        <v>0.13692614389224808</v>
+        <v>0.18</v>
       </c>
       <c r="C41" s="1">
-        <v>0.3223525557165377</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="D41" s="1">
-        <v>0.21370454836907732</v>
+        <v>0.24</v>
       </c>
       <c r="E41" s="1">
-        <v>0.16845530395506941</v>
+        <v>0.17</v>
       </c>
       <c r="F41" s="1">
-        <v>0.15856144806706762</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
@@ -1240,19 +1240,19 @@
         <v>2003</v>
       </c>
       <c r="B42" s="1">
-        <v>0.17559737132062814</v>
+        <v>0.26</v>
       </c>
       <c r="C42" s="1">
-        <v>0.26396888065291796</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="D42" s="1">
-        <v>0.28440910832372146</v>
+        <v>0.26</v>
       </c>
       <c r="E42" s="1">
-        <v>0.10867325248260086</v>
+        <v>0.04</v>
       </c>
       <c r="F42" s="1">
-        <v>0.16735138722013154</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
@@ -1260,19 +1260,19 @@
         <v>2004</v>
       </c>
       <c r="B43" s="1">
-        <v>0.11656318804857088</v>
+        <v>0.13</v>
       </c>
       <c r="C43" s="1">
-        <v>0.34649310740090022</v>
+        <v>0.35</v>
       </c>
       <c r="D43" s="1">
-        <v>0.22058929006165356</v>
+        <v>0.17</v>
       </c>
       <c r="E43" s="1">
-        <v>0.15308319414440844</v>
+        <v>0.17</v>
       </c>
       <c r="F43" s="1">
-        <v>0.16327122034446684</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
@@ -1280,19 +1280,19 @@
         <v>2005</v>
       </c>
       <c r="B44" s="1">
-        <v>0.29130003451723196</v>
+        <v>0.33</v>
       </c>
       <c r="C44" s="1">
-        <v>0.20845380602886218</v>
+        <v>0.22</v>
       </c>
       <c r="D44" s="1">
-        <v>0.24319408576675089</v>
+        <v>0.19</v>
       </c>
       <c r="E44" s="1">
-        <v>0.10139377492749711</v>
+        <v>0.1</v>
       </c>
       <c r="F44" s="1">
-        <v>0.15565829875965775</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
@@ -1300,19 +1300,19 @@
         <v>2006</v>
       </c>
       <c r="B45" s="1">
-        <v>0.17378943401458008</v>
+        <v>0.13</v>
       </c>
       <c r="C45" s="1">
-        <v>0.44310400311915998</v>
+        <v>0.47</v>
       </c>
       <c r="D45" s="1">
-        <v>0.12202857899607067</v>
+        <v>0.11</v>
       </c>
       <c r="E45" s="1">
-        <v>0.10794490629803498</v>
+        <v>0.11</v>
       </c>
       <c r="F45" s="1">
-        <v>0.15313307757215433</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
@@ -1320,19 +1320,19 @@
         <v>2007</v>
       </c>
       <c r="B46" s="1">
-        <v>0.29494304913089414</v>
+        <v>0.31</v>
       </c>
       <c r="C46" s="1">
-        <v>0.27030556011313372</v>
+        <v>0.26</v>
       </c>
       <c r="D46" s="1">
-        <v>0.29789336301534852</v>
+        <v>0.3</v>
       </c>
       <c r="E46" s="1">
-        <v>5.6866362237872191E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F46" s="1">
-        <v>7.9991665502751386E-2</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
@@ -1340,19 +1340,19 @@
         <v>2008</v>
       </c>
       <c r="B47" s="1">
-        <v>0.15719383467693107</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="C47" s="1">
-        <v>0.48261936385604981</v>
+        <v>0.47</v>
       </c>
       <c r="D47" s="1">
-        <v>0.15742942667254647</v>
+        <v>0.19</v>
       </c>
       <c r="E47" s="1">
-        <v>0.13349240104766419</v>
+        <v>0.13</v>
       </c>
       <c r="F47" s="1">
-        <v>6.9264973746808511E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
@@ -1360,19 +1360,19 @@
         <v>2009</v>
       </c>
       <c r="B48" s="1">
-        <v>0.44001473230597615</v>
+        <v>0.43</v>
       </c>
       <c r="C48" s="1">
-        <v>0.2309951305691863</v>
+        <v>0.25</v>
       </c>
       <c r="D48" s="1">
-        <v>0.23306619081046798</v>
+        <v>0.19</v>
       </c>
       <c r="E48" s="1">
-        <v>5.7017288422212722E-2</v>
+        <v>0.08</v>
       </c>
       <c r="F48" s="1">
-        <v>3.890665789215686E-2</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
@@ -1380,19 +1380,19 @@
         <v>2010</v>
       </c>
       <c r="B49" s="1">
-        <v>0.12980583859345357</v>
+        <v>0.15</v>
       </c>
       <c r="C49" s="1">
-        <v>0.65546551932387531</v>
+        <v>0.6</v>
       </c>
       <c r="D49" s="1">
-        <v>0.1094997421972731</v>
+        <v>0.1</v>
       </c>
       <c r="E49" s="1">
-        <v>8.8012107325337832E-2</v>
+        <v>0.12</v>
       </c>
       <c r="F49" s="1">
-        <v>1.7216792560060146E-2</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
@@ -1400,19 +1400,19 @@
         <v>2011</v>
       </c>
       <c r="B50" s="1">
-        <v>0.16683643320476538</v>
+        <v>0.22</v>
       </c>
       <c r="C50" s="1">
-        <v>0.26476908572410013</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="D50" s="1">
-        <v>0.42639858371804779</v>
+        <v>0.36</v>
       </c>
       <c r="E50" s="1">
-        <v>5.9414432314405664E-2</v>
+        <v>0.08</v>
       </c>
       <c r="F50" s="1">
-        <v>8.2581465038681023E-2</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.2">
@@ -1420,19 +1420,19 @@
         <v>2012</v>
       </c>
       <c r="B51" s="1">
-        <v>0.24518177687880049</v>
+        <v>0.25</v>
       </c>
       <c r="C51" s="1">
-        <v>0.30102246638076818</v>
+        <v>0.3</v>
       </c>
       <c r="D51" s="1">
-        <v>0.19471465360281584</v>
+        <v>0.24</v>
       </c>
       <c r="E51" s="1">
-        <v>0.22549722877700887</v>
+        <v>0.19</v>
       </c>
       <c r="F51" s="1">
-        <v>3.3583874360606725E-2</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
@@ -1440,19 +1440,19 @@
         <v>2013</v>
       </c>
       <c r="B52" s="1">
-        <v>0.31363392417068797</v>
+        <v>0.32</v>
       </c>
       <c r="C52" s="1">
-        <v>0.33211434355058794</v>
+        <v>0.33</v>
       </c>
       <c r="D52" s="1">
-        <v>0.17074350572048677</v>
+        <v>0.1</v>
       </c>
       <c r="E52" s="1">
-        <v>6.8376043453476698E-2</v>
+        <v>0.11</v>
       </c>
       <c r="F52" s="1">
-        <v>0.11513218310476059</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
@@ -1460,19 +1460,19 @@
         <v>2014</v>
       </c>
       <c r="B53" s="1">
-        <v>0.24758527252471607</v>
+        <v>0.36</v>
       </c>
       <c r="C53" s="1">
-        <v>0.47288376119353948</v>
+        <v>0.4</v>
       </c>
       <c r="D53" s="1">
-        <v>0.19021033099286042</v>
+        <v>0.18</v>
       </c>
       <c r="E53" s="1">
-        <v>6.0415918441601449E-2</v>
+        <v>0.06</v>
       </c>
       <c r="F53" s="1">
-        <v>2.8904716847282574E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
@@ -1480,19 +1480,19 @@
         <v>2015</v>
       </c>
       <c r="B54" s="1">
-        <v>0.2835518410668425</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="C54" s="1">
-        <v>0.32487096700378953</v>
+        <v>0.36</v>
       </c>
       <c r="D54" s="1">
-        <v>0.26637112543949804</v>
+        <v>0.3</v>
       </c>
       <c r="E54" s="1">
-        <v>7.4436261345148469E-2</v>
+        <v>0.04</v>
       </c>
       <c r="F54" s="1">
-        <v>5.0769805144721514E-2</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
@@ -1500,19 +1500,19 @@
         <v>2016</v>
       </c>
       <c r="B55" s="1">
-        <v>0.19411653442855126</v>
+        <v>0.23</v>
       </c>
       <c r="C55" s="1">
-        <v>0.47071895480064535</v>
+        <v>0.4</v>
       </c>
       <c r="D55" s="1">
-        <v>0.20669711490020326</v>
+        <v>0.27</v>
       </c>
       <c r="E55" s="1">
-        <v>0.10592929251814907</v>
+        <v>0.09</v>
       </c>
       <c r="F55" s="1">
-        <v>2.25381033524511E-2</v>
+        <v>0.01</v>
       </c>
     </row>
   </sheetData>
@@ -1553,27 +1553,21 @@
         <v>1963</v>
       </c>
       <c r="B2" s="2">
-        <v>0.50585595867297928</v>
+        <v>0.54</v>
       </c>
       <c r="C2" s="2">
-        <v>0.32286803900291705</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="D2" s="2">
-        <v>9.443361266323079E-2</v>
+        <v>0.11</v>
       </c>
       <c r="E2" s="2">
-        <v>6.1271083950806993E-2</v>
+        <v>0.06</v>
       </c>
       <c r="F2" s="2">
-        <v>1.5571305710065944E-2</v>
+        <v>0.01</v>
       </c>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
@@ -1584,27 +1578,21 @@
         <v>1964</v>
       </c>
       <c r="B3" s="2">
-        <v>0.387727960590803</v>
+        <v>0.32</v>
       </c>
       <c r="C3" s="2">
-        <v>0.40598525352282427</v>
+        <v>0.38</v>
       </c>
       <c r="D3" s="2">
-        <v>0.14264781148678413</v>
+        <v>0.21</v>
       </c>
       <c r="E3" s="2">
-        <v>4.299851055322465E-2</v>
+        <v>0.03</v>
       </c>
       <c r="F3" s="2">
-        <v>2.0640463846363945E-2</v>
+        <v>0.06</v>
       </c>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
@@ -1615,27 +1603,21 @@
         <v>1965</v>
       </c>
       <c r="B4" s="2">
-        <v>0.33045756488650163</v>
+        <v>0.33</v>
       </c>
       <c r="C4" s="2">
-        <v>0.41378943882374963</v>
+        <v>0.41</v>
       </c>
       <c r="D4" s="2">
-        <v>0.17379631087385403</v>
+        <v>0.18</v>
       </c>
       <c r="E4" s="2">
-        <v>6.468127721065603E-2</v>
+        <v>0.06</v>
       </c>
       <c r="F4" s="2">
-        <v>1.7275408205238561E-2</v>
+        <v>0.02</v>
       </c>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
       <c r="P4" s="2"/>
@@ -1646,27 +1628,21 @@
         <v>1966</v>
       </c>
       <c r="B5" s="2">
-        <v>0.30963598947181814</v>
+        <v>0.35</v>
       </c>
       <c r="C5" s="2">
-        <v>0.27770732738203158</v>
+        <v>0.25</v>
       </c>
       <c r="D5" s="2">
-        <v>0.29072324482565554</v>
+        <v>0.3</v>
       </c>
       <c r="E5" s="2">
-        <v>9.0269627850229447E-2</v>
+        <v>0.1</v>
       </c>
       <c r="F5" s="2">
-        <v>3.1663810470265223E-2</v>
+        <v>0</v>
       </c>
       <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
@@ -1677,27 +1653,21 @@
         <v>1967</v>
       </c>
       <c r="B6" s="2">
-        <v>0.60371473492515115</v>
+        <v>0.65</v>
       </c>
       <c r="C6" s="2">
-        <v>0.17778882269422605</v>
+        <v>0.15</v>
       </c>
       <c r="D6" s="2">
-        <v>0.12288175534319119</v>
+        <v>0.12</v>
       </c>
       <c r="E6" s="2">
-        <v>6.8868282196197825E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F6" s="2">
-        <v>2.6746404841233772E-2</v>
+        <v>0.01</v>
       </c>
       <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
       <c r="P6" s="2"/>
@@ -1708,27 +1678,21 @@
         <v>1968</v>
       </c>
       <c r="B7" s="2">
-        <v>0.51474464739960735</v>
+        <v>0.5</v>
       </c>
       <c r="C7" s="2">
-        <v>0.36349867087730864</v>
+        <v>0.32</v>
       </c>
       <c r="D7" s="2">
-        <v>6.4573706441155593E-2</v>
+        <v>0.06</v>
       </c>
       <c r="E7" s="2">
-        <v>4.1325502218729347E-2</v>
+        <v>0.09</v>
       </c>
       <c r="F7" s="2">
-        <v>1.5857473063199245E-2</v>
+        <v>0.03</v>
       </c>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
       <c r="P7" s="2"/>
@@ -1739,27 +1703,21 @@
         <v>1969</v>
       </c>
       <c r="B8" s="2">
-        <v>0.28522385869697076</v>
+        <v>0.34</v>
       </c>
       <c r="C8" s="2">
-        <v>0.51059290233985455</v>
+        <v>0.51</v>
       </c>
       <c r="D8" s="2">
-        <v>0.16416984438041576</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="E8" s="2">
-        <v>2.6723013887234932E-2</v>
+        <v>0</v>
       </c>
       <c r="F8" s="2">
-        <v>1.3290380695523943E-2</v>
+        <v>0.01</v>
       </c>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
       <c r="P8" s="2"/>
@@ -1770,27 +1728,21 @@
         <v>1970</v>
       </c>
       <c r="B9" s="2">
-        <v>0.55394054939735404</v>
+        <v>0.5</v>
       </c>
       <c r="C9" s="2">
-        <v>0.18388672829957245</v>
+        <v>0.22</v>
       </c>
       <c r="D9" s="2">
-        <v>0.21028196233380217</v>
+        <v>0.25</v>
       </c>
       <c r="E9" s="2">
-        <v>4.5679076512287552E-2</v>
+        <v>0.03</v>
       </c>
       <c r="F9" s="2">
-        <v>6.2116834569837399E-3</v>
+        <v>0</v>
       </c>
       <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
       <c r="P9" s="2"/>
@@ -1801,27 +1753,21 @@
         <v>1971</v>
       </c>
       <c r="B10" s="2">
-        <v>0.62724202826983622</v>
+        <v>0.69</v>
       </c>
       <c r="C10" s="2">
-        <v>0.28707680366495714</v>
+        <v>0.23</v>
       </c>
       <c r="D10" s="2">
-        <v>4.50728209643236E-2</v>
+        <v>0.03</v>
       </c>
       <c r="E10" s="2">
-        <v>3.2445543982120392E-2</v>
+        <v>0.03</v>
       </c>
       <c r="F10" s="2">
-        <v>8.1628031187625481E-3</v>
+        <v>0.02</v>
       </c>
       <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
       <c r="P10" s="2"/>
@@ -1832,27 +1778,21 @@
         <v>1972</v>
       </c>
       <c r="B11" s="2">
-        <v>0.26444376620457288</v>
+        <v>0.26</v>
       </c>
       <c r="C11" s="2">
-        <v>0.5689628063436174</v>
+        <v>0.59</v>
       </c>
       <c r="D11" s="2">
-        <v>0.13031589013887795</v>
+        <v>0.11</v>
       </c>
       <c r="E11" s="2">
-        <v>2.1289780745744925E-2</v>
+        <v>0.02</v>
       </c>
       <c r="F11" s="2">
-        <v>1.4987756567186747E-2</v>
+        <v>0.02</v>
       </c>
       <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
       <c r="P11" s="2"/>
@@ -1863,27 +1803,21 @@
         <v>1973</v>
       </c>
       <c r="B12" s="2">
-        <v>0.61897563089027152</v>
+        <v>0.67</v>
       </c>
       <c r="C12" s="2">
-        <v>0.15467750500589975</v>
+        <v>0.15</v>
       </c>
       <c r="D12" s="2">
-        <v>0.18421585623829081</v>
+        <v>0.13</v>
       </c>
       <c r="E12" s="2">
-        <v>3.7409477327016501E-2</v>
+        <v>0.02</v>
       </c>
       <c r="F12" s="2">
-        <v>4.7215305385214373E-3</v>
+        <v>0.03</v>
       </c>
       <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
       <c r="P12" s="2"/>
@@ -1894,27 +1828,21 @@
         <v>1974</v>
       </c>
       <c r="B13" s="2">
-        <v>0.53387680870469068</v>
+        <v>0.52</v>
       </c>
       <c r="C13" s="2">
-        <v>0.36379833918420007</v>
+        <v>0.38</v>
       </c>
       <c r="D13" s="2">
-        <v>4.8065509382688991E-2</v>
+        <v>0.01</v>
       </c>
       <c r="E13" s="2">
-        <v>4.7138069101397298E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F13" s="2">
-        <v>7.1212736270229249E-3</v>
+        <v>0.02</v>
       </c>
       <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
       <c r="P13" s="2"/>
@@ -1925,27 +1853,21 @@
         <v>1975</v>
       </c>
       <c r="B14" s="2">
-        <v>0.2309783233383931</v>
+        <v>0.21</v>
       </c>
       <c r="C14" s="2">
-        <v>0.52327026075589311</v>
+        <v>0.52</v>
       </c>
       <c r="D14" s="2">
-        <v>0.20531273563769378</v>
+        <v>0.21</v>
       </c>
       <c r="E14" s="2">
-        <v>2.2695818969802273E-2</v>
+        <v>0.03</v>
       </c>
       <c r="F14" s="2">
-        <v>1.7742861298217803E-2</v>
+        <v>0.03</v>
       </c>
       <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
       <c r="P14" s="2"/>
@@ -1956,27 +1878,21 @@
         <v>1976</v>
       </c>
       <c r="B15" s="2">
-        <v>0.74962529560584534</v>
+        <v>0.75</v>
       </c>
       <c r="C15" s="2">
-        <v>0.10529535544964523</v>
+        <v>0.1</v>
       </c>
       <c r="D15" s="2">
-        <v>0.11208235268742317</v>
+        <v>0.13</v>
       </c>
       <c r="E15" s="2">
-        <v>2.933157126511074E-2</v>
+        <v>0.02</v>
       </c>
       <c r="F15" s="2">
-        <v>3.665424991975533E-3</v>
+        <v>0</v>
       </c>
       <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
       <c r="P15" s="2"/>
@@ -1987,27 +1903,21 @@
         <v>1977</v>
       </c>
       <c r="B16" s="2">
-        <v>0.44420542166621496</v>
+        <v>0.49</v>
       </c>
       <c r="C16" s="2">
-        <v>0.47005329286505948</v>
+        <v>0.41</v>
       </c>
       <c r="D16" s="2">
-        <v>4.8933867017480502E-2</v>
+        <v>0.03</v>
       </c>
       <c r="E16" s="2">
-        <v>2.8568777686991138E-2</v>
+        <v>0.05</v>
       </c>
       <c r="F16" s="2">
-        <v>8.2386407642539624E-3</v>
+        <v>0.02</v>
       </c>
       <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
       <c r="P16" s="2"/>
@@ -2018,27 +1928,21 @@
         <v>1978</v>
       </c>
       <c r="B17" s="2">
-        <v>0.50635021881244524</v>
+        <v>0.51</v>
       </c>
       <c r="C17" s="2">
-        <v>0.34665722087216139</v>
+        <v>0.38</v>
       </c>
       <c r="D17" s="2">
-        <v>0.13008199205444526</v>
+        <v>0.1</v>
       </c>
       <c r="E17" s="2">
-        <v>9.014609428781982E-3</v>
+        <v>0.01</v>
       </c>
       <c r="F17" s="2">
-        <v>7.8959588321659557E-3</v>
+        <v>0</v>
       </c>
       <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
       <c r="P17" s="2"/>
@@ -2049,27 +1953,21 @@
         <v>1979</v>
       </c>
       <c r="B18" s="2">
-        <v>0.62188495087114193</v>
+        <v>0.64</v>
       </c>
       <c r="C18" s="2">
-        <v>0.25603347901184592</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="D18" s="2">
-        <v>8.5825371714254056E-2</v>
+        <v>0.06</v>
       </c>
       <c r="E18" s="2">
-        <v>3.439387765589122E-2</v>
+        <v>0.01</v>
       </c>
       <c r="F18" s="2">
-        <v>1.8623207468668034E-3</v>
+        <v>0</v>
       </c>
       <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
       <c r="P18" s="2"/>
@@ -2080,27 +1978,21 @@
         <v>1980</v>
       </c>
       <c r="B19" s="2">
-        <v>0.48743445097279137</v>
+        <v>0.48</v>
       </c>
       <c r="C19" s="2">
-        <v>0.40249577547306331</v>
+        <v>0.39</v>
       </c>
       <c r="D19" s="2">
-        <v>8.2328937521496393E-2</v>
+        <v>0.08</v>
       </c>
       <c r="E19" s="2">
-        <v>2.1794669055752131E-2</v>
+        <v>0.05</v>
       </c>
       <c r="F19" s="2">
-        <v>5.9461669768968752E-3</v>
+        <v>0</v>
       </c>
       <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
-      <c r="L19" s="2"/>
-      <c r="M19" s="2"/>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
       <c r="P19" s="2"/>
@@ -2111,27 +2003,21 @@
         <v>1981</v>
       </c>
       <c r="B20" s="2">
-        <v>0.39678863445687063</v>
+        <v>0.51</v>
       </c>
       <c r="C20" s="2">
-        <v>0.34827232234713917</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="D20" s="2">
-        <v>0.22136362675921437</v>
+        <v>0.17</v>
       </c>
       <c r="E20" s="2">
-        <v>2.623740814681472E-2</v>
+        <v>0.03</v>
       </c>
       <c r="F20" s="2">
-        <v>7.3380082899611159E-3</v>
+        <v>0.01</v>
       </c>
       <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-      <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
       <c r="P20" s="2"/>
@@ -2142,27 +2028,21 @@
         <v>1982</v>
       </c>
       <c r="B21" s="2">
-        <v>0.84698219029561683</v>
+        <v>0.82</v>
       </c>
       <c r="C21" s="2">
-        <v>8.7099177070089615E-2</v>
+        <v>0.06</v>
       </c>
       <c r="D21" s="2">
-        <v>4.6572243357458222E-2</v>
+        <v>0.08</v>
       </c>
       <c r="E21" s="2">
-        <v>1.6729278340309399E-2</v>
+        <v>0.04</v>
       </c>
       <c r="F21" s="2">
-        <v>2.6171109365257963E-3</v>
+        <v>0</v>
       </c>
       <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
-      <c r="L21" s="2"/>
-      <c r="M21" s="2"/>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
       <c r="P21" s="2"/>
@@ -2173,27 +2053,21 @@
         <v>1983</v>
       </c>
       <c r="B22" s="2">
-        <v>0.24999136707161979</v>
+        <v>0.27</v>
       </c>
       <c r="C22" s="2">
-        <v>0.68728148245438803</v>
+        <v>0.65</v>
       </c>
       <c r="D22" s="2">
-        <v>3.8887983372363648E-2</v>
+        <v>0.06</v>
       </c>
       <c r="E22" s="2">
-        <v>1.6966392263010693E-2</v>
+        <v>0.01</v>
       </c>
       <c r="F22" s="2">
-        <v>6.8727748386178721E-3</v>
+        <v>0.01</v>
       </c>
       <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
       <c r="P22" s="2"/>
@@ -2204,27 +2078,21 @@
         <v>1984</v>
       </c>
       <c r="B23" s="2">
-        <v>0.38238602330470667</v>
+        <v>0.34</v>
       </c>
       <c r="C23" s="2">
-        <v>0.29768911711554596</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="D23" s="2">
-        <v>0.2980282575790531</v>
+        <v>0.35</v>
       </c>
       <c r="E23" s="2">
-        <v>1.6046251756041355E-2</v>
+        <v>0.03</v>
       </c>
       <c r="F23" s="2">
-        <v>5.8503502446528429E-3</v>
+        <v>0</v>
       </c>
       <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
       <c r="P23" s="2"/>
@@ -2235,27 +2103,21 @@
         <v>1985</v>
       </c>
       <c r="B24" s="2">
-        <v>0.60709887692226838</v>
+        <v>0.62</v>
       </c>
       <c r="C24" s="2">
-        <v>0.22931767022608804</v>
+        <v>0.25</v>
       </c>
       <c r="D24" s="2">
-        <v>7.407249097762586E-2</v>
+        <v>0.05</v>
       </c>
       <c r="E24" s="2">
-        <v>8.5309405770775559E-2</v>
+        <v>0.08</v>
       </c>
       <c r="F24" s="2">
-        <v>4.2015561032422346E-3</v>
+        <v>0</v>
       </c>
       <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
       <c r="P24" s="2"/>
@@ -2266,27 +2128,21 @@
         <v>1986</v>
       </c>
       <c r="B25" s="2">
-        <v>0.55209508486166725</v>
+        <v>0.54</v>
       </c>
       <c r="C25" s="2">
-        <v>0.35109915061971525</v>
+        <v>0.37</v>
       </c>
       <c r="D25" s="2">
-        <v>5.9332874212580405E-2</v>
+        <v>0.06</v>
       </c>
       <c r="E25" s="2">
-        <v>2.1734528408308279E-2</v>
+        <v>0.02</v>
       </c>
       <c r="F25" s="2">
-        <v>1.573836189772879E-2</v>
+        <v>0.01</v>
       </c>
       <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
       <c r="P25" s="2"/>
@@ -2297,27 +2153,21 @@
         <v>1987</v>
       </c>
       <c r="B26" s="2">
-        <v>0.50751884503245859</v>
+        <v>0.51</v>
       </c>
       <c r="C26" s="2">
-        <v>0.33982796034403168</v>
+        <v>0.31</v>
       </c>
       <c r="D26" s="2">
-        <v>0.12848098409565409</v>
+        <v>0.16</v>
       </c>
       <c r="E26" s="2">
-        <v>1.8528252180305915E-2</v>
+        <v>0.01</v>
       </c>
       <c r="F26" s="2">
-        <v>5.6439583475496932E-3</v>
+        <v>0.01</v>
       </c>
       <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
-      <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
       <c r="P26" s="2"/>
@@ -2328,27 +2178,21 @@
         <v>1988</v>
       </c>
       <c r="B27" s="2">
-        <v>0.70125367152500784</v>
+        <v>0.79</v>
       </c>
       <c r="C27" s="2">
-        <v>0.18774853816177295</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="D27" s="2">
-        <v>9.0243421690475084E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E27" s="2">
-        <v>1.7904927643317897E-2</v>
+        <v>0</v>
       </c>
       <c r="F27" s="2">
-        <v>2.8494409794261764E-3</v>
+        <v>0</v>
       </c>
       <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
-      <c r="K27" s="2"/>
-      <c r="L27" s="2"/>
-      <c r="M27" s="2"/>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
       <c r="P27" s="2"/>
@@ -2359,27 +2203,21 @@
         <v>1989</v>
       </c>
       <c r="B28" s="2">
-        <v>0.33013298328709412</v>
+        <v>0.39</v>
       </c>
       <c r="C28" s="2">
-        <v>0.5571898637880307</v>
+        <v>0.52</v>
       </c>
       <c r="D28" s="2">
-        <v>7.8539297455509263E-2</v>
+        <v>0.08</v>
       </c>
       <c r="E28" s="2">
-        <v>2.672748534256817E-2</v>
+        <v>0.01</v>
       </c>
       <c r="F28" s="2">
-        <v>7.41037012679765E-3</v>
+        <v>0</v>
       </c>
       <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
-      <c r="K28" s="2"/>
-      <c r="L28" s="2"/>
-      <c r="M28" s="2"/>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
       <c r="P28" s="2"/>
@@ -2390,27 +2228,21 @@
         <v>1990</v>
       </c>
       <c r="B29" s="2">
-        <v>0.55940085414235963</v>
+        <v>0.54</v>
       </c>
       <c r="C29" s="2">
-        <v>0.24368441809768862</v>
+        <v>0.23</v>
       </c>
       <c r="D29" s="2">
-        <v>0.17166188266817117</v>
+        <v>0.18</v>
       </c>
       <c r="E29" s="2">
-        <v>1.8545284625702239E-2</v>
+        <v>0.03</v>
       </c>
       <c r="F29" s="2">
-        <v>6.7075604660784853E-3</v>
+        <v>0.02</v>
       </c>
       <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
-      <c r="L29" s="2"/>
-      <c r="M29" s="2"/>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
       <c r="P29" s="2"/>
@@ -2421,27 +2253,21 @@
         <v>1991</v>
       </c>
       <c r="B30" s="2">
-        <v>0.53634098316623202</v>
+        <v>0.5</v>
       </c>
       <c r="C30" s="2">
-        <v>0.34871937125310704</v>
+        <v>0.34</v>
       </c>
       <c r="D30" s="2">
-        <v>7.5045157195575432E-2</v>
+        <v>0.09</v>
       </c>
       <c r="E30" s="2">
-        <v>3.5759829219983094E-2</v>
+        <v>0.06</v>
       </c>
       <c r="F30" s="2">
-        <v>4.1346591651024748E-3</v>
+        <v>0.01</v>
       </c>
       <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
-      <c r="K30" s="2"/>
-      <c r="L30" s="2"/>
-      <c r="M30" s="2"/>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
       <c r="P30" s="2"/>
@@ -2452,27 +2278,21 @@
         <v>1992</v>
       </c>
       <c r="B31" s="2">
-        <v>0.72073937032872726</v>
+        <v>0.75</v>
       </c>
       <c r="C31" s="2">
-        <v>0.21349701276409652</v>
+        <v>0.18</v>
       </c>
       <c r="D31" s="2">
-        <v>5.0638236575611562E-2</v>
+        <v>0.06</v>
       </c>
       <c r="E31" s="2">
-        <v>1.0802501249171332E-2</v>
+        <v>0.01</v>
       </c>
       <c r="F31" s="2">
-        <v>4.3228790823934072E-3</v>
+        <v>0</v>
       </c>
       <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
-      <c r="J31" s="2"/>
-      <c r="K31" s="2"/>
-      <c r="L31" s="2"/>
-      <c r="M31" s="2"/>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
       <c r="P31" s="2"/>
@@ -2483,27 +2303,21 @@
         <v>1993</v>
       </c>
       <c r="B32" s="2">
-        <v>0.45950611139220393</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="C32" s="2">
-        <v>0.45028363414562095</v>
+        <v>0.37</v>
       </c>
       <c r="D32" s="2">
-        <v>6.9227523338636951E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E32" s="2">
-        <v>1.7448064854602031E-2</v>
+        <v>0</v>
       </c>
       <c r="F32" s="2">
-        <v>3.5346662689361478E-3</v>
+        <v>0</v>
       </c>
       <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
-      <c r="K32" s="2"/>
-      <c r="L32" s="2"/>
-      <c r="M32" s="2"/>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
       <c r="P32" s="2"/>
@@ -2514,27 +2328,21 @@
         <v>1994</v>
       </c>
       <c r="B33" s="2">
-        <v>0.2785758227621935</v>
+        <v>0.34</v>
       </c>
       <c r="C33" s="2">
-        <v>0.35072710332874824</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="D33" s="2">
-        <v>0.32338739690940566</v>
+        <v>0.33</v>
       </c>
       <c r="E33" s="2">
-        <v>3.9420549414475342E-2</v>
+        <v>0.02</v>
       </c>
       <c r="F33" s="2">
-        <v>7.8891275851772757E-3</v>
+        <v>0.03</v>
       </c>
       <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
-      <c r="K33" s="2"/>
-      <c r="L33" s="2"/>
-      <c r="M33" s="2"/>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
       <c r="P33" s="2"/>
@@ -2545,27 +2353,21 @@
         <v>1995</v>
       </c>
       <c r="B34" s="2">
-        <v>0.62767380467073008</v>
+        <v>0.66</v>
       </c>
       <c r="C34" s="2">
-        <v>0.15229911087847695</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="D34" s="2">
-        <v>0.12730068213350249</v>
+        <v>0.15</v>
       </c>
       <c r="E34" s="2">
-        <v>8.0636083762401806E-2</v>
+        <v>0.08</v>
       </c>
       <c r="F34" s="2">
-        <v>1.2090318554888662E-2</v>
+        <v>0.04</v>
       </c>
       <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
-      <c r="J34" s="2"/>
-      <c r="K34" s="2"/>
-      <c r="L34" s="2"/>
-      <c r="M34" s="2"/>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
       <c r="P34" s="2"/>
@@ -2576,27 +2378,21 @@
         <v>1996</v>
       </c>
       <c r="B35" s="2">
-        <v>0.37128590530636219</v>
+        <v>0.39</v>
       </c>
       <c r="C35" s="2">
-        <v>0.43587743669356038</v>
+        <v>0.46</v>
       </c>
       <c r="D35" s="2">
-        <v>8.1071707125251607E-2</v>
+        <v>0.09</v>
       </c>
       <c r="E35" s="2">
-        <v>6.7911404864687927E-2</v>
+        <v>0.03</v>
       </c>
       <c r="F35" s="2">
-        <v>4.3853546010137884E-2</v>
+        <v>0.03</v>
       </c>
       <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
-      <c r="I35" s="2"/>
-      <c r="J35" s="2"/>
-      <c r="K35" s="2"/>
-      <c r="L35" s="2"/>
-      <c r="M35" s="2"/>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
       <c r="P35" s="2"/>
@@ -2607,27 +2403,21 @@
         <v>1997</v>
       </c>
       <c r="B36" s="2">
-        <v>0.28205448136031247</v>
+        <v>0.24</v>
       </c>
       <c r="C36" s="2">
-        <v>0.33541971805888654</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="D36" s="2">
-        <v>0.28429211372077373</v>
+        <v>0.36</v>
       </c>
       <c r="E36" s="2">
-        <v>5.3054871316791097E-2</v>
+        <v>0.05</v>
       </c>
       <c r="F36" s="2">
-        <v>4.517881554323621E-2</v>
+        <v>0.06</v>
       </c>
       <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
-      <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
-      <c r="L36" s="2"/>
-      <c r="M36" s="2"/>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
       <c r="P36" s="2"/>
@@ -2638,27 +2428,21 @@
         <v>1998</v>
       </c>
       <c r="B37" s="2">
-        <v>0.46963240660838818</v>
+        <v>0.5</v>
       </c>
       <c r="C37" s="2">
-        <v>0.20293216854346796</v>
+        <v>0.25</v>
       </c>
       <c r="D37" s="2">
-        <v>0.15162187605040603</v>
+        <v>0.13</v>
       </c>
       <c r="E37" s="2">
-        <v>0.15088450541956727</v>
+        <v>0.11</v>
       </c>
       <c r="F37" s="2">
-        <v>2.4929043378170458E-2</v>
+        <v>0.01</v>
       </c>
       <c r="G37" s="2"/>
-      <c r="H37" s="2"/>
-      <c r="I37" s="2"/>
-      <c r="J37" s="2"/>
-      <c r="K37" s="2"/>
-      <c r="L37" s="2"/>
-      <c r="M37" s="2"/>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
       <c r="P37" s="2"/>
@@ -2669,27 +2453,21 @@
         <v>1999</v>
       </c>
       <c r="B38" s="2">
-        <v>0.4643295934351544</v>
+        <v>0.51</v>
       </c>
       <c r="C38" s="2">
-        <v>0.31312678117309167</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="D38" s="2">
-        <v>9.1601063700774865E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E38" s="2">
-        <v>7.3637513757132733E-2</v>
+        <v>0.09</v>
       </c>
       <c r="F38" s="2">
-        <v>5.7305047933846255E-2</v>
+        <v>0.05</v>
       </c>
       <c r="G38" s="2"/>
-      <c r="H38" s="2"/>
-      <c r="I38" s="2"/>
-      <c r="J38" s="2"/>
-      <c r="K38" s="2"/>
-      <c r="L38" s="2"/>
-      <c r="M38" s="2"/>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
       <c r="P38" s="2"/>
@@ -2700,27 +2478,21 @@
         <v>2000</v>
       </c>
       <c r="B39" s="2">
-        <v>0.27556560222392656</v>
+        <v>0.3</v>
       </c>
       <c r="C39" s="2">
-        <v>0.42919716748264308</v>
+        <v>0.45</v>
       </c>
       <c r="D39" s="2">
-        <v>0.1911834834152851</v>
+        <v>0.1</v>
       </c>
       <c r="E39" s="2">
-        <v>5.6191677166017487E-2</v>
+        <v>0.08</v>
       </c>
       <c r="F39" s="2">
-        <v>4.7862069712127725E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="G39" s="2"/>
-      <c r="H39" s="2"/>
-      <c r="I39" s="2"/>
-      <c r="J39" s="2"/>
-      <c r="K39" s="2"/>
-      <c r="L39" s="2"/>
-      <c r="M39" s="2"/>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
       <c r="P39" s="2"/>
@@ -2731,27 +2503,21 @@
         <v>2001</v>
       </c>
       <c r="B40" s="2">
-        <v>0.40077235403199907</v>
+        <v>0.34</v>
       </c>
       <c r="C40" s="2">
-        <v>0.24740868000121907</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="D40" s="2">
-        <v>0.22554358001183272</v>
+        <v>0.23</v>
       </c>
       <c r="E40" s="2">
-        <v>9.5919147183943287E-2</v>
+        <v>0.12</v>
       </c>
       <c r="F40" s="2">
-        <v>3.0356238771005965E-2</v>
+        <v>0.03</v>
       </c>
       <c r="G40" s="2"/>
-      <c r="H40" s="2"/>
-      <c r="I40" s="2"/>
-      <c r="J40" s="2"/>
-      <c r="K40" s="2"/>
-      <c r="L40" s="2"/>
-      <c r="M40" s="2"/>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
       <c r="P40" s="2"/>
@@ -2762,27 +2528,21 @@
         <v>2002</v>
       </c>
       <c r="B41" s="2">
-        <v>0.26347063281779032</v>
+        <v>0.26</v>
       </c>
       <c r="C41" s="2">
-        <v>0.36446776634617711</v>
+        <v>0.3</v>
       </c>
       <c r="D41" s="2">
-        <v>0.17653624469658738</v>
+        <v>0.2</v>
       </c>
       <c r="E41" s="2">
-        <v>0.12876211011143271</v>
+        <v>0.15</v>
       </c>
       <c r="F41" s="2">
-        <v>6.6763246028012466E-2</v>
+        <v>0.09</v>
       </c>
       <c r="G41" s="2"/>
-      <c r="H41" s="2"/>
-      <c r="I41" s="2"/>
-      <c r="J41" s="2"/>
-      <c r="K41" s="2"/>
-      <c r="L41" s="2"/>
-      <c r="M41" s="2"/>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
       <c r="P41" s="2"/>
@@ -2793,27 +2553,21 @@
         <v>2003</v>
       </c>
       <c r="B42" s="2">
-        <v>0.39004329077196814</v>
+        <v>0.51</v>
       </c>
       <c r="C42" s="2">
-        <v>0.23927421758055556</v>
+        <v>0.19</v>
       </c>
       <c r="D42" s="2">
-        <v>0.21072379968820584</v>
+        <v>0.13</v>
       </c>
       <c r="E42" s="2">
-        <v>8.8905668504266219E-2</v>
+        <v>0.1</v>
       </c>
       <c r="F42" s="2">
-        <v>7.1053023455004208E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="G42" s="2"/>
-      <c r="H42" s="2"/>
-      <c r="I42" s="2"/>
-      <c r="J42" s="2"/>
-      <c r="K42" s="2"/>
-      <c r="L42" s="2"/>
-      <c r="M42" s="2"/>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
       <c r="P42" s="2"/>
@@ -2824,27 +2578,21 @@
         <v>2004</v>
       </c>
       <c r="B43" s="2">
-        <v>0.26683518964092784</v>
+        <v>0.21</v>
       </c>
       <c r="C43" s="2">
-        <v>0.39554773824498823</v>
+        <v>0.38</v>
       </c>
       <c r="D43" s="2">
-        <v>0.1489242550684359</v>
+        <v>0.15</v>
       </c>
       <c r="E43" s="2">
-        <v>0.13356506146657104</v>
+        <v>0.16</v>
       </c>
       <c r="F43" s="2">
-        <v>5.5127755579076988E-2</v>
+        <v>0.1</v>
       </c>
       <c r="G43" s="2"/>
-      <c r="H43" s="2"/>
-      <c r="I43" s="2"/>
-      <c r="J43" s="2"/>
-      <c r="K43" s="2"/>
-      <c r="L43" s="2"/>
-      <c r="M43" s="2"/>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
       <c r="P43" s="2"/>
@@ -2855,27 +2603,21 @@
         <v>2005</v>
       </c>
       <c r="B44" s="2">
-        <v>0.51014736349544831</v>
+        <v>0.46</v>
       </c>
       <c r="C44" s="2">
-        <v>0.18221908051280553</v>
+        <v>0.19</v>
       </c>
       <c r="D44" s="2">
-        <v>0.18524958118392298</v>
+        <v>0.26</v>
       </c>
       <c r="E44" s="2">
-        <v>6.7421924405901279E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F44" s="2">
-        <v>5.4962050401921772E-2</v>
+        <v>0.02</v>
       </c>
       <c r="G44" s="2"/>
-      <c r="H44" s="2"/>
-      <c r="I44" s="2"/>
-      <c r="J44" s="2"/>
-      <c r="K44" s="2"/>
-      <c r="L44" s="2"/>
-      <c r="M44" s="2"/>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
       <c r="P44" s="2"/>
@@ -2886,27 +2628,21 @@
         <v>2006</v>
       </c>
       <c r="B45" s="2">
-        <v>0.32501892748565764</v>
+        <v>0.3</v>
       </c>
       <c r="C45" s="2">
-        <v>0.44933693751390508</v>
+        <v>0.52</v>
       </c>
       <c r="D45" s="2">
-        <v>0.10120683204790448</v>
+        <v>0.08</v>
       </c>
       <c r="E45" s="2">
-        <v>9.1005430288342487E-2</v>
+        <v>0.08</v>
       </c>
       <c r="F45" s="2">
-        <v>3.3431872664190211E-2</v>
+        <v>0.02</v>
       </c>
       <c r="G45" s="2"/>
-      <c r="H45" s="2"/>
-      <c r="I45" s="2"/>
-      <c r="J45" s="2"/>
-      <c r="K45" s="2"/>
-      <c r="L45" s="2"/>
-      <c r="M45" s="2"/>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
       <c r="P45" s="2"/>
@@ -2917,27 +2653,21 @@
         <v>2007</v>
       </c>
       <c r="B46" s="2">
-        <v>0.51438307481285439</v>
+        <v>0.49</v>
       </c>
       <c r="C46" s="2">
-        <v>0.21843429180035995</v>
+        <v>0.26</v>
       </c>
       <c r="D46" s="2">
-        <v>0.19728776195080416</v>
+        <v>0.18</v>
       </c>
       <c r="E46" s="2">
-        <v>3.6896421363793862E-2</v>
+        <v>0.03</v>
       </c>
       <c r="F46" s="2">
-        <v>3.2998450072187685E-2</v>
+        <v>0.04</v>
       </c>
       <c r="G46" s="2"/>
-      <c r="H46" s="2"/>
-      <c r="I46" s="2"/>
-      <c r="J46" s="2"/>
-      <c r="K46" s="2"/>
-      <c r="L46" s="2"/>
-      <c r="M46" s="2"/>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
       <c r="P46" s="2"/>
@@ -2948,27 +2678,21 @@
         <v>2008</v>
       </c>
       <c r="B47" s="2">
-        <v>0.33598394634845757</v>
+        <v>0.27</v>
       </c>
       <c r="C47" s="2">
-        <v>0.42848747810264159</v>
+        <v>0.44</v>
       </c>
       <c r="D47" s="2">
-        <v>0.11804628296186552</v>
+        <v>0.15</v>
       </c>
       <c r="E47" s="2">
-        <v>9.8644095118863934E-2</v>
+        <v>0.13</v>
       </c>
       <c r="F47" s="2">
-        <v>1.8838197468171385E-2</v>
+        <v>0.01</v>
       </c>
       <c r="G47" s="2"/>
-      <c r="H47" s="2"/>
-      <c r="I47" s="2"/>
-      <c r="J47" s="2"/>
-      <c r="K47" s="2"/>
-      <c r="L47" s="2"/>
-      <c r="M47" s="2"/>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
       <c r="P47" s="2"/>
@@ -2979,27 +2703,21 @@
         <v>2009</v>
       </c>
       <c r="B48" s="2">
-        <v>0.68119482723793223</v>
+        <v>0.7</v>
       </c>
       <c r="C48" s="2">
-        <v>0.14847144490639183</v>
+        <v>0.16</v>
       </c>
       <c r="D48" s="2">
-        <v>0.12238371779183263</v>
+        <v>0.09</v>
       </c>
       <c r="E48" s="2">
-        <v>2.7707294632742799E-2</v>
+        <v>0.03</v>
       </c>
       <c r="F48" s="2">
-        <v>2.0242715431100448E-2</v>
+        <v>0.02</v>
       </c>
       <c r="G48" s="2"/>
-      <c r="H48" s="2"/>
-      <c r="I48" s="2"/>
-      <c r="J48" s="2"/>
-      <c r="K48" s="2"/>
-      <c r="L48" s="2"/>
-      <c r="M48" s="2"/>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
       <c r="P48" s="2"/>
@@ -3010,27 +2728,21 @@
         <v>2010</v>
       </c>
       <c r="B49" s="2">
-        <v>0.24800572748791716</v>
+        <v>0.21</v>
       </c>
       <c r="C49" s="2">
-        <v>0.59358135685093716</v>
+        <v>0.63</v>
       </c>
       <c r="D49" s="2">
-        <v>8.3507701009932822E-2</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E49" s="2">
-        <v>6.0527582072561079E-2</v>
+        <v>0.06</v>
       </c>
       <c r="F49" s="2">
-        <v>1.4377632578651845E-2</v>
+        <v>0.03</v>
       </c>
       <c r="G49" s="2"/>
-      <c r="H49" s="2"/>
-      <c r="I49" s="2"/>
-      <c r="J49" s="2"/>
-      <c r="K49" s="2"/>
-      <c r="L49" s="2"/>
-      <c r="M49" s="2"/>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
       <c r="P49" s="2"/>
@@ -3041,27 +2753,21 @@
         <v>2011</v>
       </c>
       <c r="B50" s="2">
-        <v>0.33583924186928288</v>
+        <v>0.35</v>
       </c>
       <c r="C50" s="2">
-        <v>0.24258809977932466</v>
+        <v>0.24</v>
       </c>
       <c r="D50" s="2">
-        <v>0.34450187644215874</v>
+        <v>0.34</v>
       </c>
       <c r="E50" s="2">
-        <v>4.4087660820035041E-2</v>
+        <v>0.04</v>
       </c>
       <c r="F50" s="2">
-        <v>3.2983121089198708E-2</v>
+        <v>0.03</v>
       </c>
       <c r="G50" s="2"/>
-      <c r="H50" s="2"/>
-      <c r="I50" s="2"/>
-      <c r="J50" s="2"/>
-      <c r="K50" s="2"/>
-      <c r="L50" s="2"/>
-      <c r="M50" s="2"/>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
       <c r="P50" s="2"/>
@@ -3072,27 +2778,21 @@
         <v>2012</v>
       </c>
       <c r="B51" s="2">
-        <v>0.4409241204638617</v>
+        <v>0.45</v>
       </c>
       <c r="C51" s="2">
-        <v>0.28472722349813068</v>
+        <v>0.22</v>
       </c>
       <c r="D51" s="2">
-        <v>0.1139050112713635</v>
+        <v>0.13</v>
       </c>
       <c r="E51" s="2">
-        <v>0.1427428334984418</v>
+        <v>0.16</v>
       </c>
       <c r="F51" s="2">
-        <v>1.7700811268202211E-2</v>
+        <v>0.04</v>
       </c>
       <c r="G51" s="2"/>
-      <c r="H51" s="2"/>
-      <c r="I51" s="2"/>
-      <c r="J51" s="2"/>
-      <c r="K51" s="2"/>
-      <c r="L51" s="2"/>
-      <c r="M51" s="2"/>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
       <c r="P51" s="2"/>
@@ -3103,27 +2803,21 @@
         <v>2013</v>
       </c>
       <c r="B52" s="2">
-        <v>0.5520792545121006</v>
+        <v>0.49</v>
       </c>
       <c r="C52" s="2">
-        <v>0.26522889559682844</v>
+        <v>0.25</v>
       </c>
       <c r="D52" s="2">
-        <v>9.6211992045104472E-2</v>
+        <v>0.1</v>
       </c>
       <c r="E52" s="2">
-        <v>3.7902677365225949E-2</v>
+        <v>0.06</v>
       </c>
       <c r="F52" s="2">
-        <v>4.8577180480740556E-2</v>
+        <v>0.1</v>
       </c>
       <c r="G52" s="2"/>
-      <c r="H52" s="2"/>
-      <c r="I52" s="2"/>
-      <c r="J52" s="2"/>
-      <c r="K52" s="2"/>
-      <c r="L52" s="2"/>
-      <c r="M52" s="2"/>
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
       <c r="P52" s="2"/>
@@ -3134,27 +2828,21 @@
         <v>2014</v>
       </c>
       <c r="B53" s="2">
-        <v>0.45487396031449079</v>
+        <v>0.31</v>
       </c>
       <c r="C53" s="2">
-        <v>0.35735574906539158</v>
+        <v>0.42</v>
       </c>
       <c r="D53" s="2">
-        <v>0.12851336885432607</v>
+        <v>0.19</v>
       </c>
       <c r="E53" s="2">
-        <v>4.1607471383481864E-2</v>
+        <v>0.06</v>
       </c>
       <c r="F53" s="2">
-        <v>1.7649450382309691E-2</v>
+        <v>0.02</v>
       </c>
       <c r="G53" s="2"/>
-      <c r="H53" s="2"/>
-      <c r="I53" s="2"/>
-      <c r="J53" s="2"/>
-      <c r="K53" s="2"/>
-      <c r="L53" s="2"/>
-      <c r="M53" s="2"/>
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
       <c r="P53" s="2"/>
@@ -3165,27 +2853,21 @@
         <v>2015</v>
       </c>
       <c r="B54" s="2">
-        <v>0.50346151861802935</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="C54" s="2">
-        <v>0.27358352717007517</v>
+        <v>0.19</v>
       </c>
       <c r="D54" s="2">
-        <v>0.15694581124054222</v>
+        <v>0.17</v>
       </c>
       <c r="E54" s="2">
-        <v>4.9117404930783037E-2</v>
+        <v>0.06</v>
       </c>
       <c r="F54" s="2">
-        <v>1.6891738040570259E-2</v>
+        <v>0.01</v>
       </c>
       <c r="G54" s="2"/>
-      <c r="H54" s="2"/>
-      <c r="I54" s="2"/>
-      <c r="J54" s="2"/>
-      <c r="K54" s="2"/>
-      <c r="L54" s="2"/>
-      <c r="M54" s="2"/>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
       <c r="P54" s="2"/>
@@ -3196,27 +2878,21 @@
         <v>2016</v>
       </c>
       <c r="B55" s="2">
-        <v>0.33478136432138761</v>
+        <v>0.31</v>
       </c>
       <c r="C55" s="2">
-        <v>0.41645951320722752</v>
+        <v>0.39</v>
       </c>
       <c r="D55" s="2">
-        <v>0.15036298139256946</v>
+        <v>0.16</v>
       </c>
       <c r="E55" s="2">
-        <v>7.6411038660254907E-2</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="F55" s="2">
-        <v>2.1985102418560633E-2</v>
+        <v>0</v>
       </c>
       <c r="G55" s="2"/>
-      <c r="H55" s="2"/>
-      <c r="I55" s="2"/>
-      <c r="J55" s="2"/>
-      <c r="K55" s="2"/>
-      <c r="L55" s="2"/>
-      <c r="M55" s="2"/>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
       <c r="P55" s="2"/>

</xml_diff>